<commit_message>
Update database naming conventions and enhance documentation in CLAUDE.md
- Revised database naming conventions in the admin portal to clearly differentiate between the admin portal database (`erb_admin_portal`) and per-domain document databases (`erb_<domain>`).
- Updated `CLAUDE.md` to emphasize the importance of maintaining distinct category boundaries in naming to avoid confusion.
- Refactored `server.js` and related scripts to implement the new naming conventions consistently across the codebase.
- Adjusted SQL and JSON files to align with the updated database structure, ensuring clarity and maintainability.
- Improved overall documentation for better understanding of the admin portal's architecture and database interactions.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -8,6 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ERBVersions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ERBCustomizations" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -182,6 +184,11 @@
         <t>Full name is computed from the first and last name of the customer</t>
       </text>
     </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Identifier for the customers.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -475,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -484,6 +491,8 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -494,40 +503,49 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>EmailAddress</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>FirstName</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>LastName</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>FullName</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>EmailAddress</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>FirstName</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>LastName</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>FullName</t>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>From_field_Customer</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>cust0001</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>CUST0001</t>
-        </is>
+          <t>jane-smith-email-com</t>
+        </is>
+      </c>
+      <c r="B2" s="3">
+        <f>SUBSTITUTE($C2, "@", "-")</f>
+        <v/>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -536,7 +554,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Jane</t>
+          <t>Bobby</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -548,17 +566,18 @@
         <f>$E2 &amp; ", " &amp; $D2</f>
         <v/>
       </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>cust0002</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>CUST0002</t>
-        </is>
+          <t>john-doe-email-com</t>
+        </is>
+      </c>
+      <c r="B3" s="3">
+        <f>SUBSTITUTE($C3, "@", "-")</f>
+        <v/>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -567,7 +586,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>John</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -579,17 +598,18 @@
         <f>$E3 &amp; ", " &amp; $D3</f>
         <v/>
       </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>cust0003</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>CUST0003</t>
-        </is>
+          <t>emily-jones-email-com</t>
+        </is>
+      </c>
+      <c r="B4" s="3">
+        <f>SUBSTITUTE($C4, "@", "-")</f>
+        <v/>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -598,7 +618,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Emily</t>
+          <t>Mary</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -610,9 +630,356 @@
         <f>$E4 &amp; ", " &amp; $D4</f>
         <v/>
       </c>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ERBVersionId</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>BaseId</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Message</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>CommitDate</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>IsPublished</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ERBCustomizationId</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>SQLCode</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>SQLTarget</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>CustomizationType</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>03a-customize-schema-sql</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>03a-customize-schema.sql</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Customize Schema</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-- ============================================================================
+-- CUSTOMIZE SCHEMA - User-defined tables and schema modifications
+-- ============================================================================
+-- This file is for YOUR custom schema changes that should persist across
+-- regeneration of the base ERB files.
+--
+-- USE THIS FILE FOR:
+--   - Additional tables not defined in the rulebook
+--   - Extra columns on existing tables (ALTER TABLE)
+--   - Custom indexes for performance tuning
+--   - Custom constraints or triggers
+--
+-- IMPORTANT:
+--   - This file runs AFTER 01-drop-and-create-tables.sql
+--   - The base tables already exist when this runs
+--   - This file will NOT be overwritten by ERB regeneration
+--
+-- ============================================================================
+-- Your custom schema changes go here:
+</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Postgres</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>03b-customize-functions-sql</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>03b-customize-functions.sql</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Customize Functions</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-- ============================================================================
+-- CUSTOMIZE FUNCTIONS - User-defined calculation functions
+-- ============================================================================
+-- This file is for YOUR custom PostgreSQL functions that should persist
+-- across regeneration of the base ERB files.
+--
+-- IMPORTANT:
+--   - This file runs AFTER 02-create-functions.sql
+--   - Base ERB calc functions already exist when this runs
+--   - This file will NOT be overwritten by ERB regeneration
+--
+-- ============================================================================
+-- Your custom functions go here:
+</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Postgres</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Functions</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>03c-customize-views-sql</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>03c-customize-views.sql</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Customize Views</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-- ============================================================================
+-- CUSTOMIZE VIEWS - User-defined views and view extensions
+-- ============================================================================
+-- This file is for YOUR custom views that should persist across
+-- regeneration of the base ERB files.
+--
+-- IMPORTANT:
+--   - This file runs AFTER 03-create-views.sql
+--   - All base vw_* views already exist when this runs
+--   - This file will NOT be overwritten by ERB regeneration
+--
+-- ============================================================================
+-- Your custom views go here:
+</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Postgres</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Views</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>03d-customize-rls-sql</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>03d-customize-rls.sql</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Customize Policies (RLS)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-- ============================================================================
+-- CUSTOMIZE POLICIES - User-defined Row Level Security policies
+-- ============================================================================
+-- This file is for YOUR custom RLS policies that should persist across
+-- regeneration of the base ERB files.
+--
+-- IMPORTANT:
+--   - This file runs AFTER 04-create-policies.sql
+--   - Base RLS policies already exist when this runs
+--   - This file will NOT be overwritten by ERB regeneration
+--
+-- ============================================================================
+-- Your custom policies go here:
+</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Postgres</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>RLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>03e-customize-data-sql</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>03e-customize-data.sql</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Customize Data (Seeds / Migrations)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-- ============================================================================
+-- CUSTOMIZE DATA - User-defined seed data and data migrations
+-- ============================================================================
+-- This file is for YOUR custom seed data that should persist across
+-- regeneration of the base ERB files.
+--
+-- IMPORTANT:
+--   - This file runs AFTER 05-insert-data.sql
+--   - Base seed data already exists when this runs
+--   - This file will NOT be overwritten by ERB regeneration
+--
+-- ============================================================================
+-- Your custom data inserts go here:
+</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Postgres</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update customer rulebook and SQL scripts for consistency and clarity
- Refactored customer-fullname-rulebook.json to streamline schema definitions and improve clarity in field descriptions.
- Adjusted SQL scripts to enhance comments and ensure accurate descriptions for tables and views.
- Modified the full name calculation function to concatenate first and last names correctly.
- Updated seed data for customers to reflect accurate first names.
- Revised binary Excel files for customer and job search examples.

These changes improve the overall structure and readability of the rulebook and associated SQL scripts.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Bobby</t>
+          <t>Bob</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="F2" s="3">
-        <f>$E2 &amp; ", " &amp; $D2</f>
+        <f>$D2 &amp; " " &amp; $E2</f>
         <v/>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="F3" s="3">
-        <f>$E3 &amp; ", " &amp; $D3</f>
+        <f>$D3 &amp; " " &amp; $E3</f>
         <v/>
       </c>
     </row>
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="F4" s="3">
-        <f>$E4 &amp; ", " &amp; $D4</f>
+        <f>$D4 &amp; " " &amp; $E4</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance active-domain handling and UI interactions
- Updated CLAUDE.md to clarify the role of `active-domain.txt` as a CLI and conversation scratchpad, emphasizing that it should not be used to infer user intent.
- Refactored `RoleTopBar` to ensure domain switching only affects the URL, without mutating `active-domain.txt`, aligning with the updated doctrine.
- Improved error handling in `server.js` for rulebook updates, ensuring non-empty and valid JSON is required before saving.
- Enhanced `ExplorerScreen` and related components to consistently pass the current domain, ensuring accurate data handling across UI interactions.
- Updated rulebook JSON files to correct and add fields, improving clarity and functionality.

These changes aim to streamline user interactions and maintain the integrity of the active domain context across the application.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__meta__" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -186,6 +187,41 @@
 </comments>
 </file>
 
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>ERB Rulebook</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>The metadata key (e.g. 'tagline', 'motif_palette', 'substrates'). Unique within the table.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Identifier for this metadata entry. Mirrors MetaKey so the row is addressable by Name like every other table.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>How to interpret the value columns: 'string' (use StringValue), 'object' (parse JsonValue as JSON object), 'array' (parse JsonValue as JSON array).</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Plain string value. Populated when ValueType == 'string'; null otherwise.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>JSON-encoded value. Populated when ValueType == 'object' or 'array'; null when ValueType == 'string'.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -612,4 +648,230 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MetaKey</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ValueType</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>StringValue</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>JsonValue</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>tagline</t>
+        </is>
+      </c>
+      <c r="B2" s="3">
+        <f>$A2</f>
+        <v/>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>One table. One calculated field. That's the whole demo.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>motif</t>
+        </is>
+      </c>
+      <c r="B3" s="3">
+        <f>$A3</f>
+        <v/>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>description_rich</t>
+        </is>
+      </c>
+      <c r="B4" s="3">
+        <f>$A4</f>
+        <v/>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>The smallest non-trivial Effortless rulebook. **One** entity (`Customers`), three rows, and a single calculated field — `FullName = FirstName &amp; " " &amp; LastName`. The argument is the simplicity itself: this much logic, lifted out of application code and into the rulebook, propagates to every substrate. Postgres view, Python class, Excel cell, OWL ontology — all four compute the same answer the same way, from the same rulebook JSON, with zero glue code.
+This is the rulebook to point a skeptic at when *every other demo feels like too much*.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>use_cases</t>
+        </is>
+      </c>
+      <c r="B5" s="3">
+        <f>$A5</f>
+        <v/>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>["**Edit `FirstName` on any row and watch `FullName` recompute in every substrate.** No application code reads this field — the rulebook IS the field.", "**Compare the Postgres view, the Python class, and the Excel cell** for the same row. They all compute `FullName` from the same formula declared once in the rulebook.", "**Try adding a calculated field of your own** — say `Initials = LEFT(FirstName, 1) &amp; LEFT(LastName, 1)`. Run `effortless build`. Every substrate now has it."]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>signature_rows</t>
+        </is>
+      </c>
+      <c r="B6" s="3">
+        <f>$A6</f>
+        <v/>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>[{"entity": "Customers", "ids": ["jane-smith-email-com", "john-doe-email-com", "emily-jones-email-com"]}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>journal_seed</t>
+        </is>
+      </c>
+      <c r="B7" s="3">
+        <f>$A7</f>
+        <v/>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Three customers. One calculated field. The whole point of ERB, on a napkin.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>substrates</t>
+        </is>
+      </c>
+      <c r="B8" s="3">
+        <f>$A8</f>
+        <v/>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>[{"key": "postgres", "important": true, "chip_label": "Postgres"}, {"key": "python", "important": true, "chip_label": "Python"}, {"key": "excel", "important": false, "chip_label": "Excel"}, {"key": "owl", "important": false, "chip_label": "OWL"}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>motif_palette</t>
+        </is>
+      </c>
+      <c r="B9" s="3">
+        <f>$A9</f>
+        <v/>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>{"primary": "#2b4a6a", "accent": "#e6a544", "ink": "#0d1b2a"}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Implement rulebook validation and enhance error handling
- Introduced a pre-flight validation function for proposed rulebooks, leveraging a Python transpiler to catch syntax errors and ensure integrity before saving.
- Updated error handling in the API responses to include detailed transpiler output when validation fails, improving user feedback.
- Enhanced the ExplorerScreen to display validation errors more clearly, ensuring users are informed of issues without losing unsaved changes.
- Adjusted rulebook JSON files to reflect new validation requirements and updated calculated fields, enhancing overall functionality.

These changes aim to improve the robustness of rulebook management and provide clearer feedback to users during the editing process.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -170,15 +170,20 @@
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
+        <t>dsfdfds</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
         <t>First Name of the customer - used to make the full name</t>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
+    <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <t>Last Name of the customer - used to make the full name</t>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
+    <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <t>Full name is computed from the first and last name of the customer</t>
       </text>
@@ -511,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -520,6 +525,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -540,15 +546,20 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Initials</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>FirstName</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>LastName</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>FullName</t>
         </is>
@@ -569,18 +580,23 @@
           <t>jane.smith@email.com</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>LEFT(FirstName, 1) &amp; LEFT(LastName, 1)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Jane</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Smith</t>
         </is>
       </c>
-      <c r="F2" s="3">
-        <f>$D2 &amp; " " &amp; $E2</f>
+      <c r="G2" s="3">
+        <f>$E2 &amp; " " &amp; $F2</f>
         <v/>
       </c>
     </row>
@@ -599,18 +615,23 @@
           <t>john.doe@email.com</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>LEFT(FirstName, 1) &amp; LEFT(LastName, 1)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Jimmy</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Doe</t>
         </is>
       </c>
-      <c r="F3" s="3">
-        <f>$D3 &amp; " " &amp; $E3</f>
+      <c r="G3" s="3">
+        <f>$E3 &amp; " " &amp; $F3</f>
         <v/>
       </c>
     </row>
@@ -629,18 +650,23 @@
           <t>emily.jones@email.com</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>LEFT(FirstName, 1) &amp; LEFT(LastName, 1)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Mary</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Jones</t>
         </is>
       </c>
-      <c r="F4" s="3">
-        <f>$D4 &amp; " " &amp; $E4</f>
+      <c r="G4" s="3">
+        <f>$E4 &amp; " " &amp; $F4</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor domain handling and enhance API interactions
- Updated the handling of active domains across the application, ensuring that the URL serves as the source of truth for domain context.
- Refactored components to consistently utilize the new `makeDomainApi` function, which appends the current domain to API calls, improving data accuracy and reducing errors.
- Removed reliance on `active-domain.txt` for domain context in the UI, aligning with the updated doctrine that emphasizes URL-driven state management.
- Enhanced error handling in the API to provide clearer feedback when domain-related issues occur.
- Updated documentation in CLAUDE.md to reflect changes in domain management practices.

These changes aim to streamline user interactions and maintain the integrity of domain context throughout the application.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -580,10 +580,9 @@
           <t>jane.smith@email.com</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>LEFT(FirstName, 1) &amp; LEFT(LastName, 1)</t>
-        </is>
+      <c r="D2" s="3">
+        <f>LEFT($F2, 1) &amp; LEFT($E2, 1)</f>
+        <v/>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -596,7 +595,7 @@
         </is>
       </c>
       <c r="G2" s="3">
-        <f>$E2 &amp; " " &amp; $F2</f>
+        <f>$F2 &amp; " -*- " &amp; $E2</f>
         <v/>
       </c>
     </row>
@@ -615,10 +614,9 @@
           <t>john.doe@email.com</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>LEFT(FirstName, 1) &amp; LEFT(LastName, 1)</t>
-        </is>
+      <c r="D3" s="3">
+        <f>LEFT($F3, 1) &amp; LEFT($E3, 1)</f>
+        <v/>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -631,7 +629,7 @@
         </is>
       </c>
       <c r="G3" s="3">
-        <f>$E3 &amp; " " &amp; $F3</f>
+        <f>$F3 &amp; " -*- " &amp; $E3</f>
         <v/>
       </c>
     </row>
@@ -650,10 +648,9 @@
           <t>emily.jones@email.com</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>LEFT(FirstName, 1) &amp; LEFT(LastName, 1)</t>
-        </is>
+      <c r="D4" s="3">
+        <f>LEFT($F4, 1) &amp; LEFT($E4, 1)</f>
+        <v/>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -666,7 +663,7 @@
         </is>
       </c>
       <c r="G4" s="3">
-        <f>$E4 &amp; " " &amp; $F4</f>
+        <f>$F4 &amp; " -*- " &amp; $E4</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update customer rulebook and SQL functions for name calculations
- Removed unnecessary fields from the customer rulebook JSON, simplifying the structure.
- Updated the formula for calculating initials and full names in the SQL functions to reflect the new naming convention.
- Changed the seed data for customers to ensure consistency with the updated naming logic.
- Updated the Excel rulebook to align with the changes made in the JSON and SQL files.

These modifications enhance the clarity and functionality of the customer data representation across different substrates.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -581,12 +581,12 @@
         </is>
       </c>
       <c r="D2" s="3">
-        <f>LEFT($F2, 1) &amp; LEFT($E2, 1)</f>
+        <f>$E2 &amp; " " &amp; LEFT($F2, 1) &amp; "."</f>
         <v/>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Jane</t>
+          <t>Linda</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="G2" s="3">
-        <f>$F2 &amp; " -*- " &amp; $E2</f>
+        <f>$E2 &amp; " " &amp; $F2</f>
         <v/>
       </c>
     </row>
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="D3" s="3">
-        <f>LEFT($F3, 1) &amp; LEFT($E3, 1)</f>
+        <f>$E3 &amp; " " &amp; LEFT($F3, 1) &amp; "."</f>
         <v/>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -629,7 +629,7 @@
         </is>
       </c>
       <c r="G3" s="3">
-        <f>$F3 &amp; " -*- " &amp; $E3</f>
+        <f>$E3 &amp; " " &amp; $F3</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="D4" s="3">
-        <f>LEFT($F4, 1) &amp; LEFT($E4, 1)</f>
+        <f>$E4 &amp; " " &amp; LEFT($F4, 1) &amp; "."</f>
         <v/>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="G4" s="3">
-        <f>$F4 &amp; " -*- " &amp; $E4</f>
+        <f>$E4 &amp; " " &amp; $F4</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Postgres to Rulebook transpiler and enhance rulebook examples
- Introduced a new transpiler, `postgres-to-rulebook`, to refresh derived fields in the rulebook from Postgres views, ensuring data consistency.
- Updated rulebook examples for various projects to include the new command line options for the `rulebook-to-postgres` tool, enabling destructive rebuilds.
- Enhanced SQL bootstrap scripts to clarify the drop-all functionality, ensuring a clean slate for database initialization.
- Adjusted customer rulebook JSON files to reflect updated naming conventions and added new fields for better data representation.

These changes improve the integration between Postgres and the rulebook, enhancing data accuracy and management across different examples.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -586,12 +586,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Linda</t>
+          <t>Jane</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Smith</t>
+          <t>Smithy</t>
         </is>
       </c>
       <c r="G2" s="3">
@@ -620,7 +620,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Jimmy</t>
+          <t>John</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Mary</t>
+          <t>Emily</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Enhance Postgres integration and update rulebook examples
- Updated the `rulebook-to-postgres` command line options in various rulebook examples to include new parameters for destructive rebuilds, ensuring better control over database initialization.
- Introduced a new API endpoint for launching domain applications, allowing users to run the domain's `start.sh` script and retrieve the application URL.
- Added functionality for importing current Postgres data into the rulebook, enabling users to adopt the latest database state as the new seed data.
- Enhanced SQL bootstrap scripts to clarify the drop-all functionality, ensuring a clean slate for database initialization.
- Updated frontend components to support new launch and import features, improving user experience and operational clarity.

These changes improve the integration between Postgres and the rulebook, enhancing data accuracy and management across different examples.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -581,12 +581,12 @@
         </is>
       </c>
       <c r="D2" s="3">
-        <f>$E2 &amp; " " &amp; LEFT($F2, 1) &amp; "."</f>
+        <f>LEFT($E2, 1) &amp; "" &amp; LEFT($F2, 1)</f>
         <v/>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Jane</t>
+          <t>Mary</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="G2" s="3">
-        <f>$E2 &amp; " " &amp; $F2</f>
+        <f>$E2 &amp; " - " &amp; $F2</f>
         <v/>
       </c>
     </row>
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="D3" s="3">
-        <f>$E3 &amp; " " &amp; LEFT($F3, 1) &amp; "."</f>
+        <f>LEFT($E3, 1) &amp; "" &amp; LEFT($F3, 1)</f>
         <v/>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -629,7 +629,7 @@
         </is>
       </c>
       <c r="G3" s="3">
-        <f>$E3 &amp; " " &amp; $F3</f>
+        <f>$E3 &amp; " - " &amp; $F3</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="D4" s="3">
-        <f>$E4 &amp; " " &amp; LEFT($F4, 1) &amp; "."</f>
+        <f>LEFT($E4, 1) &amp; "" &amp; LEFT($F4, 1)</f>
         <v/>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="G4" s="3">
-        <f>$E4 &amp; " " &amp; $F4</f>
+        <f>$E4 &amp; " - " &amp; $F4</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor Postgres integration and introduce calculated field transpiler
- Updated the `server.js` and `server.py` files to replace the `postgres-to-rulebook` transpiler with `postgres-calculated-to-rulebook`, enhancing the handling of derived fields in the rulebook.
- Added a new Python script for the `postgres-calculated-to-rulebook` transpiler, which refreshes calculated field values from Postgres views, ensuring data consistency.
- Modified various rulebook example configurations to utilize the new transpiler, improving the clarity and functionality of the integration with Postgres.
- Adjusted customer rulebook JSON files to reflect the updated naming conventions and command line options for the new transpiler.

These changes enhance the accuracy and management of derived fields across different rulebook examples.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="G2" s="3">
-        <f>$E2 &amp; " - " &amp; $F2</f>
+        <f>$E2 &amp; " " &amp; $F2</f>
         <v/>
       </c>
     </row>
@@ -629,7 +629,7 @@
         </is>
       </c>
       <c r="G3" s="3">
-        <f>$E3 &amp; " - " &amp; $F3</f>
+        <f>$E3 &amp; " " &amp; $F3</f>
         <v/>
       </c>
     </row>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="G4" s="3">
-        <f>$E4 &amp; " - " &amp; $F4</f>
+        <f>$E4 &amp; " " &amp; $F4</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor admin portal schema handling and update rulebook examples
- Removed the mirroring of RulebookFlavors into the admin database, simplifying the schema management in `server.js`.
- Updated the `bootstrapDomainSchema` function to indicate that domain schema bootstrapping is now a no-op, as the necessary tables are generated by the effortless build transpiler.
- Adjusted API endpoints to eliminate unnecessary database write operations for rulebook entities, streamlining the data handling process.
- Modified customer rulebook JSON files to reflect updated naming conventions and improved descriptions for navigation items.
- Enhanced SQL functions for calculating customer names to align with new formatting requirements.

These changes improve the clarity and efficiency of the admin portal's schema management and enhance the user experience in the rulebook examples.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="D2" s="3">
-        <f>LEFT($E2, 1) &amp; "" &amp; LEFT($F2, 1)</f>
+        <f>LEFT($E2, 1) &amp; "" &amp; LEFT($F2, 1) &amp; ""</f>
         <v/>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="G2" s="3">
-        <f>$E2 &amp; " " &amp; $F2</f>
+        <f>$E2 &amp; " ... " &amp; $F2</f>
         <v/>
       </c>
     </row>
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="D3" s="3">
-        <f>LEFT($E3, 1) &amp; "" &amp; LEFT($F3, 1)</f>
+        <f>LEFT($E3, 1) &amp; "" &amp; LEFT($F3, 1) &amp; ""</f>
         <v/>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -629,7 +629,7 @@
         </is>
       </c>
       <c r="G3" s="3">
-        <f>$E3 &amp; " " &amp; $F3</f>
+        <f>$E3 &amp; " ... " &amp; $F3</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="D4" s="3">
-        <f>LEFT($E4, 1) &amp; "" &amp; LEFT($F4, 1)</f>
+        <f>LEFT($E4, 1) &amp; "" &amp; LEFT($F4, 1) &amp; ""</f>
         <v/>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -663,7 +663,41 @@
         </is>
       </c>
       <c r="G4" s="3">
-        <f>$E4 &amp; " " &amp; $F4</f>
+        <f>$E4 &amp; " ... " &amp; $F4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>alice-cooper</t>
+        </is>
+      </c>
+      <c r="B5" s="3">
+        <f>SUBSTITUTE($C5, "@", "-")</f>
+        <v/>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>alice@cooper.com</t>
+        </is>
+      </c>
+      <c r="D5" s="3">
+        <f>LEFT($E5, 1) &amp; "" &amp; LEFT($F5, 1) &amp; ""</f>
+        <v/>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Alice</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Dangerfields</t>
+        </is>
+      </c>
+      <c r="G5" s="3">
+        <f>$E5 &amp; " ... " &amp; $F5</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update customer rulebook and SQL functions for name formatting
- Refactored the formulas for calculating initials and full names in the customer rulebook JSON and SQL functions to align with new naming conventions.
- Updated seed data for customers to reflect accurate first and last names, ensuring consistency across the application.
- Enhanced the application launch log to provide clearer server start information and URLs for the demo app.

These changes improve the clarity and accuracy of customer data representation and enhance the user experience in the rulebook examples.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -581,12 +581,12 @@
         </is>
       </c>
       <c r="D2" s="3">
-        <f>LEFT($E2, 1) &amp; "" &amp; LEFT($F2, 1) &amp; ""</f>
+        <f>LEFT($E2, 1) &amp; LEFT($F2, 1)</f>
         <v/>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Mary</t>
+          <t>Jane</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="G2" s="3">
-        <f>$E2 &amp; " ... " &amp; $F2</f>
+        <f>$F2 &amp; " " &amp; $E2</f>
         <v/>
       </c>
     </row>
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="D3" s="3">
-        <f>LEFT($E3, 1) &amp; "" &amp; LEFT($F3, 1) &amp; ""</f>
+        <f>LEFT($E3, 1) &amp; LEFT($F3, 1)</f>
         <v/>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -629,7 +629,7 @@
         </is>
       </c>
       <c r="G3" s="3">
-        <f>$E3 &amp; " ... " &amp; $F3</f>
+        <f>$F3 &amp; " " &amp; $E3</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="D4" s="3">
-        <f>LEFT($E4, 1) &amp; "" &amp; LEFT($F4, 1) &amp; ""</f>
+        <f>LEFT($E4, 1) &amp; LEFT($F4, 1)</f>
         <v/>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="G4" s="3">
-        <f>$E4 &amp; " ... " &amp; $F4</f>
+        <f>$F4 &amp; " " &amp; $E4</f>
         <v/>
       </c>
     </row>
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="D5" s="3">
-        <f>LEFT($E5, 1) &amp; "" &amp; LEFT($F5, 1) &amp; ""</f>
+        <f>LEFT($E5, 1) &amp; LEFT($F5, 1)</f>
         <v/>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -693,11 +693,11 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Dangerfields</t>
+          <t>Cooper</t>
         </is>
       </c>
       <c r="G5" s="3">
-        <f>$E5 &amp; " ... " &amp; $F5</f>
+        <f>$F5 &amp; " " &amp; $E5</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update customer initials formatting to include versioning
- Modified the formula for calculating customer initials in the rulebook JSON and SQL functions to append "-v3" to the initials, ensuring version consistency.
- Updated customer seed data to reflect the new initials format, enhancing clarity across the application.
- Adjusted the binary rulebook file to align with the updated naming conventions.

These changes improve the representation of customer data in the rulebook examples.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="D2" s="3">
-        <f>LEFT($E2, 1) &amp; LEFT($F2, 1)</f>
+        <f>LEFT($E2, 1) &amp; LEFT($F2, 1) &amp; "-v3"</f>
         <v/>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -600,7 +600,7 @@
         </is>
       </c>
       <c r="D3" s="3">
-        <f>LEFT($E3, 1) &amp; LEFT($F3, 1)</f>
+        <f>LEFT($E3, 1) &amp; LEFT($F3, 1) &amp; "-v3"</f>
         <v/>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -630,7 +630,7 @@
         </is>
       </c>
       <c r="D4" s="3">
-        <f>LEFT($E4, 1) &amp; LEFT($F4, 1)</f>
+        <f>LEFT($E4, 1) &amp; LEFT($F4, 1) &amp; "-v3"</f>
         <v/>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="D5" s="3">
-        <f>LEFT($E5, 1) &amp; LEFT($F5, 1)</f>
+        <f>LEFT($E5, 1) &amp; LEFT($F5, 1) &amp; "-v3"</f>
         <v/>
       </c>
       <c r="E5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Refactor customer name handling and update related formulas
- Changed the representation of customer names in the HTML and JSON files to use "Name" instead of "FullName" for consistency.
- Updated SQL functions and JSON formulas to remove versioning from customer initials, simplifying the format.
- Adjusted seed data to reflect the new naming conventions and initials format, enhancing clarity across the application.

These changes improve the consistency and accuracy of customer data representation in the rulebook examples.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="D2" s="3">
-        <f>LEFT($E2, 1) &amp; LEFT($F2, 1) &amp; "-v3"</f>
+        <f>LEFT($E2, 1) &amp; LEFT($F2, 1)</f>
         <v/>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -600,7 +600,7 @@
         </is>
       </c>
       <c r="D3" s="3">
-        <f>LEFT($E3, 1) &amp; LEFT($F3, 1) &amp; "-v3"</f>
+        <f>LEFT($E3, 1) &amp; LEFT($F3, 1)</f>
         <v/>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -630,7 +630,7 @@
         </is>
       </c>
       <c r="D4" s="3">
-        <f>LEFT($E4, 1) &amp; LEFT($F4, 1) &amp; "-v3"</f>
+        <f>LEFT($E4, 1) &amp; LEFT($F4, 1)</f>
         <v/>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="D5" s="3">
-        <f>LEFT($E5, 1) &amp; LEFT($F5, 1) &amp; "-v3"</f>
+        <f>LEFT($E5, 1) &amp; LEFT($F5, 1)</f>
         <v/>
       </c>
       <c r="E5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Refactor customer management and update name formatting
- Adjusted the `CalculatedCount` in the effortless rulebook JSON to reflect the correct value.
- Updated the Rails customer management scripts to streamline database checks and ensure proper initialization.
- Modified customer name formatting in the rulebook JSON and SQL functions to include versioning in the full name representation.
- Refactored the `CustomersController` to differentiate between viewing and editing customer records, enhancing clarity in the codebase.
- Updated views to reflect changes in customer name handling, ensuring consistency across the application.

These changes improve the functionality and clarity of customer data management in the Rails application.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="B2" s="3">
-        <f>$F2 &amp; ", " &amp; $E2</f>
+        <f>$F2 &amp; ", " &amp; $E2 &amp; " - v4"</f>
         <v/>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -591,7 +591,7 @@
         </is>
       </c>
       <c r="B3" s="3">
-        <f>$F3 &amp; ", " &amp; $E3</f>
+        <f>$F3 &amp; ", " &amp; $E3 &amp; " - v4"</f>
         <v/>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>$F4 &amp; ", " &amp; $E4</f>
+        <f>$F4 &amp; ", " &amp; $E4 &amp; " - v4"</f>
         <v/>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>$F5 &amp; ", " &amp; $E5</f>
+        <f>$F5 &amp; ", " &amp; $E5 &amp; " - v4"</f>
         <v/>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Gutknecht</t>
+          <t>Gutknechts</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove deprecated HTML and Rails startup scripts; update customer name formatting and add new web application structure
- Deleted the old `index.html` and `start.sh` files to streamline the project structure.
- Updated the customer name formatting in the effortless rulebook JSON to reflect the new versioning scheme.
- Introduced a new web application structure with React, including essential files like `index.html`, `package.json`, and TypeScript configurations.
- Added new components for managing customer data, enhancing the user interface and interaction.

These changes modernize the application architecture and improve the management of customer data.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="B2" s="3">
-        <f>$F2 &amp; ", " &amp; $E2 &amp; " - v4"</f>
+        <f>$F2 &amp; ": " &amp; $E2 &amp; " - v5"</f>
         <v/>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -591,7 +591,7 @@
         </is>
       </c>
       <c r="B3" s="3">
-        <f>$F3 &amp; ", " &amp; $E3 &amp; " - v4"</f>
+        <f>$F3 &amp; ": " &amp; $E3 &amp; " - v5"</f>
         <v/>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>$F4 &amp; ", " &amp; $E4 &amp; " - v4"</f>
+        <f>$F4 &amp; ": " &amp; $E4 &amp; " - v5"</f>
         <v/>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>$F5 &amp; ", " &amp; $E5 &amp; " - v4"</f>
+        <f>$F5 &amp; ": " &amp; $E5 &amp; " - v5"</f>
         <v/>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Gutknechts</t>
+          <t>Gutknecht</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update customer name formatting and enhance database scripts
- Modified the customer name formatting in the effortless rulebook JSON and SQL functions to use a comma instead of a colon, reflecting the new versioning scheme.
- Updated the customer seed data to align with the new naming conventions, ensuring consistency across the application.
- Enhanced the development log with additional entries for better tracking of customer data processing.

These changes improve the clarity and accuracy of customer data representation in the rulebook examples.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="B2" s="3">
-        <f>$F2 &amp; ": " &amp; $E2 &amp; " - v5"</f>
+        <f>$F2 &amp; ", " &amp; $E2 &amp; " - v6"</f>
         <v/>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -591,7 +591,7 @@
         </is>
       </c>
       <c r="B3" s="3">
-        <f>$F3 &amp; ": " &amp; $E3 &amp; " - v5"</f>
+        <f>$F3 &amp; ", " &amp; $E3 &amp; " - v6"</f>
         <v/>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>$F4 &amp; ": " &amp; $E4 &amp; " - v5"</f>
+        <f>$F4 &amp; ", " &amp; $E4 &amp; " - v6"</f>
         <v/>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>$F5 &amp; ": " &amp; $E5 &amp; " - v5"</f>
+        <f>$F5 &amp; ", " &amp; $E5 &amp; " - v6"</f>
         <v/>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Gutknecht</t>
+          <t>Mary</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance domain management and sorting functionality in admin portal
- Introduced a new DomainSortBar component for improved domain sorting options, allowing users to sort domains by recently opened, alphabetical order, and least recently opened.
- Updated DeveloperDomainsScreen and ViewerDomainsScreen to utilize the DomainSortBar, enhancing user experience with better domain organization.
- Implemented last modified timestamps for domains, enabling the display of how long ago each domain was last accessed.
- Enhanced server-side logic to update domain folder timestamps when accessed, improving the accuracy of sorting and recently opened features.
- Refactored related components to ensure consistent handling of domain data and improved overall performance.

These changes aim to streamline domain management and enhance user interaction within the admin portal.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -165,22 +165,17 @@
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Thec ustomers email address</t>
+        <t>First Name of the customer - used to make the full name</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>dsfdfds</t>
+        <t>Last Name of the customer - used to make the full name</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>First Name of the customer - used to make the full name</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>Last Name of the customer - used to make the full name</t>
+        <t>dsfdfds</t>
       </text>
     </comment>
   </commentList>
@@ -511,15 +506,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -535,22 +529,17 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>EmailAddress</t>
+          <t>FirstName</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>LastName</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Initials</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>FirstName</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>LastName</t>
         </is>
       </c>
     </row>
@@ -561,27 +550,22 @@
         </is>
       </c>
       <c r="B2" s="3">
-        <f>$F2 &amp; ", " &amp; $E2</f>
+        <f>$C2 &amp; " " &amp; $D2 </f>
         <v/>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>jane.smith@email.com</t>
-        </is>
-      </c>
-      <c r="D2" s="3">
-        <f>LEFT($E2, 1) &amp; LEFT($F2, 1) &amp; "."</f>
-        <v/>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
           <t>Jane</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Smithy</t>
         </is>
+      </c>
+      <c r="E2" s="3">
+        <f>LEFT($C2, 1) &amp; LEFT($D2, 1) &amp; "."</f>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -591,27 +575,22 @@
         </is>
       </c>
       <c r="B3" s="3">
-        <f>$F3 &amp; ", " &amp; $E3</f>
+        <f>$C3 &amp; " " &amp; $D3 </f>
         <v/>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>john.doe@email.com</t>
-        </is>
-      </c>
-      <c r="D3" s="3">
-        <f>LEFT($E3, 1) &amp; LEFT($F3, 1) &amp; "."</f>
-        <v/>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>John</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Doe</t>
         </is>
+      </c>
+      <c r="E3" s="3">
+        <f>LEFT($C3, 1) &amp; LEFT($D3, 1) &amp; "."</f>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -621,27 +600,22 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>$F4 &amp; ", " &amp; $E4</f>
+        <f>$C4 &amp; " " &amp; $D4 </f>
         <v/>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>emily.jones@email.com</t>
-        </is>
-      </c>
-      <c r="D4" s="3">
-        <f>LEFT($E4, 1) &amp; LEFT($F4, 1) &amp; "."</f>
-        <v/>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
           <t>Emily</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Jones</t>
         </is>
+      </c>
+      <c r="E4" s="3">
+        <f>LEFT($C4, 1) &amp; LEFT($D4, 1) &amp; "."</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -651,27 +625,22 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>$F5 &amp; ", " &amp; $E5</f>
+        <f>$C5 &amp; " " &amp; $D5 </f>
         <v/>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>alice@cooper.com</t>
-        </is>
-      </c>
-      <c r="D5" s="3">
-        <f>LEFT($E5, 1) &amp; LEFT($F5, 1) &amp; "."</f>
-        <v/>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
           <t>Alice</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Gutknecht</t>
-        </is>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Cooper</t>
+        </is>
+      </c>
+      <c r="E5" s="3">
+        <f>LEFT($C5, 1) &amp; LEFT($D5, 1) &amp; "."</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tweaked full name and initials.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -521,7 +521,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Smithy</t>
+          <t>Smith</t>
         </is>
       </c>
       <c r="D2" s="3">
@@ -529,7 +529,7 @@
         <v/>
       </c>
       <c r="E2" s="3">
-        <f>RIGHT($B2, 1) &amp; "." &amp; RIGHT($C2, 1) &amp; "."</f>
+        <f>LEFT($B2, 1) &amp; "." &amp; LEFT($C2, 1) &amp; "."</f>
         <v/>
       </c>
     </row>
@@ -554,7 +554,7 @@
         <v/>
       </c>
       <c r="E3" s="3">
-        <f>RIGHT($B3, 1) &amp; "." &amp; RIGHT($C3, 1) &amp; "."</f>
+        <f>LEFT($B3, 1) &amp; "." &amp; LEFT($C3, 1) &amp; "."</f>
         <v/>
       </c>
     </row>
@@ -579,7 +579,7 @@
         <v/>
       </c>
       <c r="E4" s="3">
-        <f>RIGHT($B4, 1) &amp; "." &amp; RIGHT($C4, 1) &amp; "."</f>
+        <f>LEFT($B4, 1) &amp; "." &amp; LEFT($C4, 1) &amp; "."</f>
         <v/>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Gutknechts</t>
+          <t>Gutknecht</t>
         </is>
       </c>
       <c r="D5" s="3">
@@ -604,7 +604,7 @@
         <v/>
       </c>
       <c r="E5" s="3">
-        <f>RIGHT($B5, 1) &amp; "." &amp; RIGHT($C5, 1) &amp; "."</f>
+        <f>LEFT($B5, 1) &amp; "." &amp; LEFT($C5, 1) &amp; "."</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update customer full name and initials formatting across multiple files
- Adjusted the formula for calculating initials in the customer rulebook JSON and SQL functions to include a space before the period, ensuring clarity in representation.
- Updated the `FullName` calculation to format as "LastName, FirstName" in various JSON files, ensuring consistency across all substrates.
- Enhanced documentation in `rulespeak.md` and `rulespeak.html` to reflect the updated naming conventions and calculations for customer data.
- Added a new script `build-explainer.sh` to bundle the React explainer-dag, improving the build process for the application.
- Reflected changes in the application launch log to provide clearer server start information and URLs for the demo app.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -529,7 +529,7 @@
         <v/>
       </c>
       <c r="E2" s="3">
-        <f>LEFT($B2, 1) &amp; "." &amp; LEFT($C2, 1) &amp; "."</f>
+        <f>LEFT($B2, 1) &amp; ". " &amp; LEFT($C2, 1) &amp; "."</f>
         <v/>
       </c>
     </row>
@@ -554,7 +554,7 @@
         <v/>
       </c>
       <c r="E3" s="3">
-        <f>LEFT($B3, 1) &amp; "." &amp; LEFT($C3, 1) &amp; "."</f>
+        <f>LEFT($B3, 1) &amp; ". " &amp; LEFT($C3, 1) &amp; "."</f>
         <v/>
       </c>
     </row>
@@ -579,7 +579,7 @@
         <v/>
       </c>
       <c r="E4" s="3">
-        <f>LEFT($B4, 1) &amp; "." &amp; LEFT($C4, 1) &amp; "."</f>
+        <f>LEFT($B4, 1) &amp; ". " &amp; LEFT($C4, 1) &amp; "."</f>
         <v/>
       </c>
     </row>
@@ -604,7 +604,7 @@
         <v/>
       </c>
       <c r="E5" s="3">
-        <f>LEFT($B5, 1) &amp; "." &amp; LEFT($C5, 1) &amp; "."</f>
+        <f>LEFT($B5, 1) &amp; ". " &amp; LEFT($C5, 1) &amp; "."</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update customer full name formatting and related documentation
- Modified the formula for calculating the customer's full name to format as "LastName, FirstName" in the JSON and SQL scripts, ensuring consistency across the application.
- Updated the corresponding documentation in `rulespeak.md` and `rulespeak.html` to reflect the new name formatting, enhancing clarity for users.
- Adjusted references in the explainer DAG and other related files to align with the updated naming convention, improving overall usability.

These changes aim to enhance the accuracy and user experience of customer data handling within the Talisman project.
</commit_message>
<xml_diff>
--- a/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
+++ b/rulebook-examples/customer-fullname/xlsx/rulebook.xlsx
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="D2" s="3">
-        <f>$B2 &amp; " " &amp; $C2</f>
+        <f>$C2 &amp; ", " &amp; $B2</f>
         <v/>
       </c>
       <c r="E2" s="3">
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="D3" s="3">
-        <f>$B3 &amp; " " &amp; $C3</f>
+        <f>$C3 &amp; ", " &amp; $B3</f>
         <v/>
       </c>
       <c r="E3" s="3">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D4" s="3">
-        <f>$B4 &amp; " " &amp; $C4</f>
+        <f>$C4 &amp; ", " &amp; $B4</f>
         <v/>
       </c>
       <c r="E4" s="3">
@@ -600,7 +600,7 @@
         </is>
       </c>
       <c r="D5" s="3">
-        <f>$B5 &amp; " " &amp; $C5</f>
+        <f>$C5 &amp; ", " &amp; $B5</f>
         <v/>
       </c>
       <c r="E5" s="3">

</xml_diff>